<commit_message>
Font Size revision in all the plots, added 'Unclear' and 'Not Acceptable' in JBI assessments, layout revisions
</commit_message>
<xml_diff>
--- a/grade_data.xlsx
+++ b/grade_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="20">
   <si>
     <t xml:space="preserve">Outcome</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t xml:space="preserve">Quality of Life</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not Reported</t>
   </si>
   <si>
     <t xml:space="preserve">Very Low</t>
@@ -445,9 +448,11 @@
         <v>9</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -491,10 +496,10 @@
         <v>8</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>